<commit_message>
V3 Azure-only pipeline: deduped results, per-field PII columns, post-search enrichment
- Add V3 pipeline: Azure AI Search-only search (no Python regex/fuzzy)
- Strategies filter files, then enrichment queries all 13 PII fields against matched docs
- Deduplicate V3 results to one row per (customer, MD5), strategies stored as JSON list
- Add 13 per-field leaked_* columns to results table (both V2 and V3)
- Store customer's master_data PII values in leaked_* columns instead of raw snippets
- V2 vs V3 comparison output: v2_vs_v3_comparison.txt
- V3 specs, design doc, indexing/search/batch services, tests, and scripts

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/simulated_files/payroll_q1_xlsx.xlsx
+++ b/data/simulated_files/payroll_q1_xlsx.xlsx
@@ -473,10 +473,10 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>21154</v>
+        <v>21713</v>
       </c>
       <c r="F2" t="n">
-        <v>15230</v>
+        <v>15633</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -504,10 +504,10 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>24463</v>
+        <v>24447</v>
       </c>
       <c r="F3" t="n">
-        <v>17613</v>
+        <v>17601</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -535,10 +535,10 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>23885</v>
+        <v>22751</v>
       </c>
       <c r="F4" t="n">
-        <v>17197</v>
+        <v>16380</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -566,10 +566,10 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>22193</v>
+        <v>21746</v>
       </c>
       <c r="F5" t="n">
-        <v>15978</v>
+        <v>15657</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -597,10 +597,10 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>21786</v>
+        <v>23306</v>
       </c>
       <c r="F6" t="n">
-        <v>15685</v>
+        <v>16780</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Remove REST API, switch to Click CLI + Poetry + Docker
- Replace FastAPI/uvicorn with Click CLI (generate, seed, index, run, status, compare)
- Add pyproject.toml with Poetry config, delete requirements.txt
- Add Dockerfile + docker-compose.yml (SQL Server 2022 + app)
- Add README.md with Docker and local setup instructions
- Extract batch query functions to app/services/batch_query_service.py
- Relocate app/schemas/pii.py to app/models/pii.py
- Remove get_db() from database.py, delete all routers/schemas/API tests
- Fix test_batch_logging.py TestLoggingConfig to use CLI instead of deleted app.main
- Fix duplicate error message in cli.py index command

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/simulated_files/payroll_q1_xlsx.xlsx
+++ b/data/simulated_files/payroll_q1_xlsx.xlsx
@@ -473,10 +473,10 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>21713</v>
+        <v>21222</v>
       </c>
       <c r="F2" t="n">
-        <v>15633</v>
+        <v>15279</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -504,10 +504,10 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>24447</v>
+        <v>22174</v>
       </c>
       <c r="F3" t="n">
-        <v>17601</v>
+        <v>15965</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -535,10 +535,10 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>22751</v>
+        <v>25848</v>
       </c>
       <c r="F4" t="n">
-        <v>16380</v>
+        <v>18610</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -566,10 +566,10 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>21746</v>
+        <v>23446</v>
       </c>
       <c r="F5" t="n">
-        <v>15657</v>
+        <v>16881</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -597,10 +597,10 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>23306</v>
+        <v>23290</v>
       </c>
       <c r="F6" t="n">
-        <v>16780</v>
+        <v>16768</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>

</xml_diff>